<commit_message>
v11.85 LIVE: the feet read as feet; turn 30 without concrete blocks; blank-box feet corrected to 11 papers
Today and Progress read Feet / bases 8,235 (the hire agreements' component boxes) where they said
Fence blocks 216; the breakdown lists all 123 hire agreements with their feet. Race-call turn 30 is the
v11.83 take with the concrete-blocks phrase cut out. The crew print-out, gear workbook and Advanced
account now count 11 papers with the feet box blank (36629's 11 braces were missed): about 8,495 used.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/print_24Oct2026_fencing_crew/GC500_2026_fencing_gear_used_by_docket.xlsx
+++ b/03_GC500_Delivery_Control/print_24Oct2026_fencing_crew/GC500_2026_fencing_gear_used_by_docket.xlsx
@@ -100,13 +100,13 @@
     <t xml:space="preserve">Dockets with the feet box left blank</t>
   </si>
   <si>
-    <t xml:space="preserve">230 panels and 4 braces on them: about 240 feet not written.</t>
+    <t xml:space="preserve">230 panels and 15 braces on them (36629 alone has 11 braces): about 260 feet not written.</t>
   </si>
   <si>
     <t xml:space="preserve">Feet used, about</t>
   </si>
   <si>
-    <t xml:space="preserve">Written + the blank papers. The gear says the same.</t>
+    <t xml:space="preserve">Written + the blank papers. The gear says the same, with one more at the open end of each run.</t>
   </si>
   <si>
     <t xml:space="preserve">If braces actually took three feet each (not what the dockets show), add one more per brace: 1,426 more, about 9,900 in all.</t>
@@ -2833,7 +2833,7 @@
         <v>23</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>24</v>
@@ -2844,8 +2844,8 @@
         <v>25</v>
       </c>
       <c r="B22" s="6" t="n">
-        <f aca="false">B20+240</f>
-        <v>8475</v>
+        <f aca="false">B20+260</f>
+        <v>8495</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>26</v>

</xml_diff>